<commit_message>
feat: update streamlit GUI and relax VIP handling
</commit_message>
<xml_diff>
--- a/outputs/安排结果_双人配对.xlsx
+++ b/outputs/安排结果_双人配对.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,22 +468,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>F7, M1</t>
+          <t>F4, M3</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>F7(唐婉清), M1(赵浩然)</t>
+          <t>F4(wanlin zheng), M3(胡永昕)</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -492,12 +492,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>F8, M8</t>
+          <t>F2, M1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>F8(曹雅楠/原F9), M8(王景辰)</t>
+          <t>F2(ariel xiao), M1(Chengzhi Peng)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -516,22 +516,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>F1, M10</t>
+          <t>F1, M4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>F1(林雨桐), M10(陈奕辰)</t>
+          <t>F1(连璐), M4(刘泽翔)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -540,12 +540,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>F6, M5</t>
+          <t>F3, M6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F6(宋可欣), M5(周嘉铭)</t>
+          <t>F3(蒲悠儿), M6(Yong Yang)</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -564,22 +564,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>F2, M2, M9</t>
+          <t>F6, M8</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>F2(何诗涵), M2(钱宇轩), M9(冯博文)</t>
+          <t>F6(You Lai), M8(JIN XIE)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -588,12 +588,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>F4, M4</t>
+          <t>F7, M10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>F4(梁欣怡), M4(李俊熙)</t>
+          <t>F7(April Cheng), M10(沈育嘉)</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -612,19 +612,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>F3, M7</t>
+          <t>F5, M2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>F3(高若曦), M7(郑明轩)</t>
+          <t>F5(Yue Lin), M2(汪喆昊)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -636,19 +636,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>F5, M6</t>
+          <t>F8, M5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>F5(谢梦瑶), M6(吴泽宇)</t>
+          <t>F8(Ellen Wan), M5(Steven Lin)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -660,21 +660,45 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>F9, M3</t>
+          <t>F9, M7</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>F9(彭思妍/原F10), M3(孙子涵)</t>
+          <t>F9(Ye Wang), M7(张延)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>F10, M9</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>F10(胥夏), M9(Kevin Shen)</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -689,7 +713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -735,31 +759,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>单向喜欢</t>
+          <t>互相喜欢</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>M1(赵浩然)</t>
+          <t>F4(wanlin zheng)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>F7</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>F7(唐婉清)</t>
+          <t>M3(胡永昕)</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -773,22 +797,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M8(王景辰)</t>
+          <t>M1(Chengzhi Peng)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>F8</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>F8(曹雅楠/原F9)</t>
+          <t>F2(ariel xiao)</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -801,7 +825,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>互相喜欢</t>
+          <t>单向喜欢</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -811,21 +835,21 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>F1(林雨桐)</t>
+          <t>F1(连璐)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>M10(陈奕辰)</t>
+          <t>M4(刘泽翔)</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -839,22 +863,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F6</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>F6(宋可欣)</t>
+          <t>M6(Yong Yang)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>M5(周嘉铭)</t>
+          <t>F3(蒲悠儿)</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -872,22 +896,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>F6</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>M9(冯博文)</t>
+          <t>F6(You Lai)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>F2(何诗涵)</t>
+          <t>M8(JIN XIE)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -896,166 +920,34 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>互相喜欢</t>
+          <t>单向喜欢</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>F2(何诗涵)</t>
+          <t>M10(沈育嘉)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>M2(钱宇轩)</t>
+          <t>F7(April Cheng)</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>单向喜欢</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>F4(梁欣怡)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>M4(李俊熙)</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>单向喜欢</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>M7</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>M7(郑明轩)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>F3(高若曦)</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>单向喜欢</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>F5(谢梦瑶)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>M6(吴泽宇)</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>单向喜欢</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>F9</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>F9(彭思妍/原F10)</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>M3(孙子涵)</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1092,7 +984,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1102,7 +994,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.555555555555555</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4">
@@ -1112,7 +1004,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1122,7 +1014,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1133,7 +1025,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>38.5%</t>
         </is>
       </c>
     </row>

</xml_diff>